<commit_message>
Added new RDF data schemes and visual schemes for employment-table11-15, fixed XLSX spreadsheets for employment-table11-14
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/employment-table11.xlsx
+++ b/sources/table_normalization/xlsx/employment-table11.xlsx
@@ -1891,17 +1891,17 @@
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2212,7 +2212,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
@@ -2242,7 +2242,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -2256,16 +2256,16 @@
     <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="7" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="7" t="s">
         <v>8</v>
       </c>
       <c r="G6" s="8" t="s">

</xml_diff>